<commit_message>
feat: add OPSAFE_CON configuration spreadsheet and update measurement logic
</commit_message>
<xml_diff>
--- a/res/OPSAFE_CON.xlsx
+++ b/res/OPSAFE_CON.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="181">
   <si>
     <t>Захід контролю ризику</t>
   </si>
@@ -802,13 +802,13 @@
     </r>
   </si>
   <si>
-    <t>EH</t>
+    <t>НВ</t>
   </si>
   <si>
-    <t>H</t>
+    <t>В</t>
   </si>
   <si>
-    <t>M</t>
+    <t>С</t>
   </si>
   <si>
     <r>
@@ -842,7 +842,10 @@
     </r>
   </si>
   <si>
-    <t>L</t>
+    <t>H</t>
+  </si>
+  <si>
+    <t>Н</t>
   </si>
   <si>
     <r>
@@ -902,7 +905,7 @@
         <color rgb="FF000000"/>
         <sz val="12.0"/>
       </rPr>
-      <t xml:space="preserve">EH </t>
+      <t xml:space="preserve">НВ </t>
     </r>
     <r>
       <rPr>
@@ -919,7 +922,7 @@
         <color rgb="FF000000"/>
         <sz val="12.0"/>
       </rPr>
-      <t xml:space="preserve">H </t>
+      <t xml:space="preserve">В </t>
     </r>
     <r>
       <rPr>
@@ -936,7 +939,7 @@
         <color rgb="FF000000"/>
         <sz val="12.0"/>
       </rPr>
-      <t xml:space="preserve">M </t>
+      <t xml:space="preserve">С </t>
     </r>
     <r>
       <rPr>
@@ -953,7 +956,7 @@
         <color rgb="FF000000"/>
         <sz val="12.0"/>
       </rPr>
-      <t xml:space="preserve">L </t>
+      <t xml:space="preserve">Н </t>
     </r>
     <r>
       <rPr>
@@ -1886,9 +1889,7 @@
         <v>1.0</v>
       </c>
       <c r="K5" s="20"/>
-      <c r="L5" s="19">
-        <v>1.0</v>
-      </c>
+      <c r="L5" s="20"/>
       <c r="M5" s="20"/>
       <c r="N5" s="20"/>
       <c r="O5" s="19">
@@ -1906,7 +1907,7 @@
       <c r="U5" s="20"/>
       <c r="V5" s="21">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W5" s="8"/>
       <c r="X5" s="8"/>
@@ -33655,9 +33656,6 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C3:C68">
       <formula1>"Координаційні,Планувальні,Операційні,Регламентні,Нагляд та контроль,Навчання"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B3:B68">
-      <formula1>"Тактичні,Інформаційна безпека,Інженерні,Технічні,Ударно-вогневі,Розвідувально-інформаційні,Маскувальні,Індивідуального захисту,Навчальні,Імітаційні,Дезінформація"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F3:F68">
       <formula1>"плановий,передопераційний,операційний"</formula1>
     </dataValidation>
@@ -33666,6 +33664,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3:E68">
       <formula1>"уникнення ризику,зменшення ризику,розподіл ризику,перенесення ризику,прийняття ризику"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B3:B68">
+      <formula1>"Тактичні,Інформаційна безпека,Інженерні,Технічні,Ударно-вогневі,Розвідувально-інформаційні,Маскувальні,Індивідуального захисту,Навчальні,Імітаційні,Дезінформація"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
@@ -37954,18 +37955,18 @@
         <v>173</v>
       </c>
       <c r="D3" s="60" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E3" s="61" t="s">
         <v>174</v>
       </c>
       <c r="F3" s="62" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" ht="60.0" customHeight="1">
       <c r="A4" s="58" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B4" s="60" t="s">
         <v>173</v>
@@ -37977,35 +37978,35 @@
         <v>174</v>
       </c>
       <c r="E4" s="62" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F4" s="62" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" ht="60.0" customHeight="1">
       <c r="A5" s="58" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B5" s="61" t="s">
         <v>174</v>
       </c>
       <c r="C5" s="62" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D5" s="62" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E5" s="62" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F5" s="62" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="63" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G6" s="64"/>
     </row>

</xml_diff>